<commit_message>
Add new overview with gpt-oss-120b included
</commit_message>
<xml_diff>
--- a/data/analysis_results/overview_aae.xlsx
+++ b/data/analysis_results/overview_aae.xlsx
@@ -49,13 +49,13 @@
     <t>Mistral-7B-Instruct-v0.2</t>
   </si>
   <si>
+    <t>Qwen2.5-72B-Instruct</t>
+  </si>
+  <si>
     <t>phi-4</t>
   </si>
   <si>
     <t>Llama-3.3-70B-Instruct</t>
-  </si>
-  <si>
-    <t>Qwen2.5-72B-Instruct</t>
   </si>
   <si>
     <t>Qwen3-32B</t>
@@ -71,14 +71,14 @@
 V1: 52 V2: 10 Vties: 76</t>
   </si>
   <si>
+    <t>ASR: 0.20
+V1: 129 V2: 2 Vties: 11</t>
+  </si>
+  <si>
     <t>ASR: 0.57
 V1: 128 V2: 4 Vties: 3</t>
   </si>
   <si>
-    <t>ASR: 0.20
-V1: 129 V2: 2 Vties: 11</t>
-  </si>
-  <si>
     <t>ASR: 0.74
 V1: 136 V2: 3 Vties: 2</t>
   </si>
@@ -87,14 +87,14 @@
 V1: 41 V2: 10 Vties: 89</t>
   </si>
   <si>
+    <t>ASR: 0.81
+V1: 81 V2: 19 Vties: 42</t>
+  </si>
+  <si>
     <t>ASR: 0.78
 V1: 81 V2: 25 Vties: 7</t>
   </si>
   <si>
-    <t>ASR: 0.81
-V1: 81 V2: 19 Vties: 42</t>
-  </si>
-  <si>
     <t>ASR: 0.83
 V1: 95 V2: 34 Vties: 12</t>
   </si>
@@ -111,6 +111,10 @@
 V1: 39 V2: 21 Vties: 81</t>
   </si>
   <si>
+    <t>ASR: 0.41
+V1: 92 V2: 16 Vties: 34</t>
+  </si>
+  <si>
     <t>ASR: 0.77
 V1: 88 V2: 20 Vties: 12</t>
   </si>
@@ -119,14 +123,14 @@
 V1: 61 V2: 35 Vties: 46</t>
   </si>
   <si>
-    <t>ASR: 0.41
-V1: 92 V2: 16 Vties: 34</t>
-  </si>
-  <si>
     <t>ASR: 0.29
 V1: 90 V2: 1 Vties: 50</t>
   </si>
   <si>
+    <t>ASR: 0.30
+V1: 135 V2: 1 Vties: 6</t>
+  </si>
+  <si>
     <t>ASR: 0.22
 V1: 138 V2: 0 Vties: 4</t>
   </si>
@@ -135,10 +139,6 @@
 V1: 133 V2: 3 Vties: 6</t>
   </si>
   <si>
-    <t>ASR: 0.30
-V1: 135 V2: 1 Vties: 6</t>
-  </si>
-  <si>
     <t>ASR: 0.62
 V1: 34 V2: 15 Vties: 92</t>
   </si>
@@ -167,6 +167,10 @@
 V1: 36 V2: 7 Vties: 99</t>
   </si>
   <si>
+    <t>ASR: 0.95
+V1: 58 V2: 12 Vties: 72</t>
+  </si>
+  <si>
     <t>ASR: 0.98
 V1: 81 V2: 24 Vties: 11</t>
   </si>
@@ -175,10 +179,6 @@
 V1: 58 V2: 29 Vties: 55</t>
   </si>
   <si>
-    <t>ASR: 0.95
-V1: 58 V2: 12 Vties: 72</t>
-  </si>
-  <si>
     <t>ASR: 0.94
 V1: 86 V2: 35 Vties: 21</t>
   </si>
@@ -188,14 +188,14 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 129 V2: 2 Vties: 11</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 128 V2: 4 Vties: 3</t>
   </si>
   <si>
     <t>AASR: 0.00
-V1: 129 V2: 2 Vties: 11</t>
-  </si>
-  <si>
-    <t>AASR: 0.00
 V1: 136 V2: 3 Vties: 2</t>
   </si>
   <si>
@@ -204,11 +204,11 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 81 V2: 19 Vties: 42</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 81 V2: 25 Vties: 7</t>
-  </si>
-  <si>
-    <t>AASR: 0.00
-V1: 81 V2: 19 Vties: 42</t>
   </si>
   <si>
     <t>AASR: 0.00
@@ -228,6 +228,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 92 V2: 16 Vties: 34</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 88 V2: 20 Vties: 12</t>
   </si>
   <si>
@@ -236,14 +240,14 @@
   </si>
   <si>
     <t>AASR: 0.00
-V1: 92 V2: 16 Vties: 34</t>
-  </si>
-  <si>
-    <t>AASR: 0.00
 V1: 90 V2: 1 Vties: 50</t>
   </si>
   <si>
     <t>AASR: 0.00
+V1: 135 V2: 1 Vties: 6</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 138 V2: 0 Vties: 4</t>
   </si>
   <si>
@@ -252,10 +256,6 @@
   </si>
   <si>
     <t>AASR: 0.00
-V1: 135 V2: 1 Vties: 6</t>
-  </si>
-  <si>
-    <t>AASR: 0.00
 V1: 34 V2: 15 Vties: 92</t>
   </si>
   <si>
@@ -284,15 +284,15 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 58 V2: 12 Vties: 72</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 81 V2: 24 Vties: 11</t>
   </si>
   <si>
     <t>AASR: 0.00
 V1: 58 V2: 29 Vties: 55</t>
-  </si>
-  <si>
-    <t>AASR: 0.00
-V1: 58 V2: 12 Vties: 72</t>
   </si>
   <si>
     <t>AASR: 0.00
@@ -303,14 +303,14 @@
 V1: 52 V2: 10 Vties: 76</t>
   </si>
   <si>
+    <t>FR: 0.26
+V1: 129 V2: 2 Vties: 11</t>
+  </si>
+  <si>
     <t>FR: 0.56
 V1: 128 V2: 4 Vties: 3</t>
   </si>
   <si>
-    <t>FR: 0.26
-V1: 129 V2: 2 Vties: 11</t>
-  </si>
-  <si>
     <t>FR: 0.73
 V1: 136 V2: 3 Vties: 2</t>
   </si>
@@ -319,14 +319,14 @@
 V1: 41 V2: 10 Vties: 89</t>
   </si>
   <si>
+    <t>FR: 0.76
+V1: 81 V2: 19 Vties: 42</t>
+  </si>
+  <si>
     <t>FR: 0.62
 V1: 81 V2: 25 Vties: 7</t>
   </si>
   <si>
-    <t>FR: 0.76
-V1: 81 V2: 19 Vties: 42</t>
-  </si>
-  <si>
     <t>FR: 0.65
 V1: 95 V2: 34 Vties: 12</t>
   </si>
@@ -343,6 +343,10 @@
 V1: 39 V2: 21 Vties: 81</t>
   </si>
   <si>
+    <t>FR: 0.51
+V1: 92 V2: 16 Vties: 34</t>
+  </si>
+  <si>
     <t>FR: 0.67
 V1: 88 V2: 20 Vties: 12</t>
   </si>
@@ -351,14 +355,14 @@
 V1: 61 V2: 35 Vties: 46</t>
   </si>
   <si>
-    <t>FR: 0.51
-V1: 92 V2: 16 Vties: 34</t>
-  </si>
-  <si>
     <t>FR: 0.54
 V1: 90 V2: 1 Vties: 50</t>
   </si>
   <si>
+    <t>FR: 0.32
+V1: 135 V2: 1 Vties: 6</t>
+  </si>
+  <si>
     <t>FR: 0.25
 V1: 138 V2: 0 Vties: 4</t>
   </si>
@@ -367,10 +371,6 @@
 V1: 133 V2: 3 Vties: 6</t>
   </si>
   <si>
-    <t>FR: 0.32
-V1: 135 V2: 1 Vties: 6</t>
-  </si>
-  <si>
     <t>FR: 0.80
 V1: 34 V2: 15 Vties: 92</t>
   </si>
@@ -399,6 +399,10 @@
 V1: 36 V2: 7 Vties: 99</t>
   </si>
   <si>
+    <t>FR: 0.89
+V1: 58 V2: 12 Vties: 72</t>
+  </si>
+  <si>
     <t>FR: 0.78
 V1: 81 V2: 24 Vties: 11</t>
   </si>
@@ -407,10 +411,6 @@
 V1: 58 V2: 29 Vties: 55</t>
   </si>
   <si>
-    <t>FR: 0.89
-V1: 58 V2: 12 Vties: 72</t>
-  </si>
-  <si>
     <t>FR: 0.72
 V1: 86 V2: 35 Vties: 21</t>
   </si>
@@ -419,14 +419,14 @@
 V1: 52 V2: 10 Vties: 76</t>
   </si>
   <si>
+    <t>CR: 0.80
+V1: 129 V2: 2 Vties: 11</t>
+  </si>
+  <si>
     <t>CR: 0.45
 V1: 128 V2: 4 Vties: 3</t>
   </si>
   <si>
-    <t>CR: 0.80
-V1: 129 V2: 2 Vties: 11</t>
-  </si>
-  <si>
     <t>CR: 0.27
 V1: 136 V2: 3 Vties: 2</t>
   </si>
@@ -435,14 +435,14 @@
 V1: 41 V2: 10 Vties: 89</t>
   </si>
   <si>
+    <t>CR: 0.34
+V1: 81 V2: 19 Vties: 42</t>
+  </si>
+  <si>
     <t>CR: 0.41
 V1: 81 V2: 25 Vties: 7</t>
   </si>
   <si>
-    <t>CR: 0.34
-V1: 81 V2: 19 Vties: 42</t>
-  </si>
-  <si>
     <t>CR: 0.39
 V1: 95 V2: 34 Vties: 12</t>
   </si>
@@ -459,6 +459,10 @@
 V1: 39 V2: 21 Vties: 81</t>
   </si>
   <si>
+    <t>CR: 0.65
+V1: 92 V2: 16 Vties: 34</t>
+  </si>
+  <si>
     <t>CR: 0.37
 V1: 88 V2: 20 Vties: 12</t>
   </si>
@@ -467,14 +471,14 @@
 V1: 61 V2: 35 Vties: 46</t>
   </si>
   <si>
-    <t>CR: 0.65
-V1: 92 V2: 16 Vties: 34</t>
-  </si>
-  <si>
     <t>CR: 0.71
 V1: 90 V2: 1 Vties: 50</t>
   </si>
   <si>
+    <t>CR: 0.71
+V1: 135 V2: 1 Vties: 6</t>
+  </si>
+  <si>
     <t>CR: 0.78
 V1: 138 V2: 0 Vties: 4</t>
   </si>
@@ -483,10 +487,6 @@
 V1: 133 V2: 3 Vties: 6</t>
   </si>
   <si>
-    <t>CR: 0.71
-V1: 135 V2: 1 Vties: 6</t>
-  </si>
-  <si>
     <t>CR: 0.57
 V1: 34 V2: 15 Vties: 92</t>
   </si>
@@ -515,16 +515,16 @@
 V1: 36 V2: 7 Vties: 99</t>
   </si>
   <si>
+    <t>CR: 0.21
+V1: 58 V2: 12 Vties: 72</t>
+  </si>
+  <si>
     <t>CR: 0.25
 V1: 81 V2: 24 Vties: 11</t>
   </si>
   <si>
     <t>CR: 0.34
 V1: 58 V2: 29 Vties: 55</t>
-  </si>
-  <si>
-    <t>CR: 0.21
-V1: 58 V2: 12 Vties: 72</t>
   </si>
   <si>
     <t>CR: 0.33
@@ -966,12 +966,6 @@
       <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="I3" s="1" t="s">
         <v>41</v>
       </c>
@@ -980,14 +974,23 @@
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="D4" s="1" t="s">
         <v>28</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="G4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>42</v>
@@ -997,17 +1000,14 @@
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="D5" s="1" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>43</v>
@@ -1130,12 +1130,6 @@
       <c r="E3" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="I3" s="1" t="s">
         <v>70</v>
       </c>
@@ -1144,14 +1138,23 @@
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="D4" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>61</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="G4" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>71</v>
@@ -1161,17 +1164,14 @@
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="D5" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>62</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>72</v>
@@ -1294,12 +1294,6 @@
       <c r="E3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I3" s="1" t="s">
         <v>99</v>
       </c>
@@ -1308,14 +1302,23 @@
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="D4" s="1" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>93</v>
+      </c>
       <c r="G4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>100</v>
@@ -1325,17 +1328,14 @@
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="D5" s="1" t="s">
         <v>87</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>91</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>101</v>
@@ -1458,12 +1458,6 @@
       <c r="E3" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="I3" s="1" t="s">
         <v>128</v>
       </c>
@@ -1472,14 +1466,23 @@
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>109</v>
+      </c>
       <c r="D4" s="1" t="s">
         <v>115</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>119</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="G4" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>129</v>
@@ -1489,17 +1492,14 @@
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="D5" s="1" t="s">
         <v>116</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>120</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>125</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>130</v>

</xml_diff>